<commit_message>
actualiza acumulados 20/06/2026 16:27
</commit_message>
<xml_diff>
--- a/Pruebas calificadas/COLEGIO ATABANZA DIAGNOSTICA 1103_CALIFICADO.xlsx
+++ b/Pruebas calificadas/COLEGIO ATABANZA DIAGNOSTICA 1103_CALIFICADO.xlsx
@@ -807,15 +807,19 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1056,15 +1060,19 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1305,15 +1313,19 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1554,15 +1566,19 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1803,15 +1819,19 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2048,15 +2068,19 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2285,15 +2309,19 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -2534,15 +2562,19 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2783,15 +2815,19 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -3028,15 +3064,19 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3277,15 +3317,19 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -3526,15 +3570,19 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -3775,15 +3823,19 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -4024,15 +4076,19 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -4273,15 +4329,19 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -4522,15 +4582,19 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -4771,15 +4835,19 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -5020,15 +5088,19 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -5269,15 +5341,19 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -5518,15 +5594,19 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -5767,15 +5847,19 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -6016,15 +6100,19 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -6265,15 +6353,19 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -6514,15 +6606,19 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -6759,15 +6855,19 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -7008,15 +7108,19 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -7257,15 +7361,19 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -7506,15 +7614,19 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -7755,15 +7867,19 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -8004,15 +8120,19 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -8253,15 +8373,19 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -8498,15 +8622,19 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -8747,15 +8875,19 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -8996,15 +9128,19 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -9245,15 +9381,19 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -9490,15 +9630,19 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -9739,15 +9883,19 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -9988,15 +10136,19 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -10237,15 +10389,19 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -10486,15 +10642,19 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -10735,15 +10895,19 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -10984,15 +11148,19 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr"/>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -11233,15 +11401,19 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -11482,15 +11654,19 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -11731,15 +11907,19 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -11980,15 +12160,19 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr"/>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -12229,15 +12413,19 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr"/>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -12478,15 +12666,19 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -12727,15 +12919,19 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr"/>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -12976,15 +13172,19 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr"/>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -13225,15 +13425,19 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr"/>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -13474,15 +13678,19 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>111001047017</t>
+          <t>111001098817</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>ATABANZHA</t>
+          <t>COLEGIO NUEVA ROMA (IED)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">

</xml_diff>

<commit_message>
actualiza acumulados 22/06/2026 10:53
</commit_message>
<xml_diff>
--- a/Pruebas calificadas/COLEGIO ATABANZA DIAGNOSTICA 1103_CALIFICADO.xlsx
+++ b/Pruebas calificadas/COLEGIO ATABANZA DIAGNOSTICA 1103_CALIFICADO.xlsx
@@ -809,17 +809,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1062,17 +1062,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1315,17 +1315,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1568,17 +1568,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1821,17 +1821,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2070,17 +2070,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2311,17 +2311,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -2564,17 +2564,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2817,17 +2817,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -3066,17 +3066,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3319,17 +3319,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -3572,17 +3572,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -3825,17 +3825,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -4078,17 +4078,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -4331,17 +4331,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -4584,17 +4584,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -4837,17 +4837,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -5090,17 +5090,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -5343,17 +5343,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -5596,17 +5596,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -5849,17 +5849,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -6102,17 +6102,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -6355,17 +6355,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -6608,17 +6608,17 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -6857,17 +6857,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -7110,17 +7110,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -7363,17 +7363,17 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -7616,17 +7616,17 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -7869,17 +7869,17 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -8122,17 +8122,17 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -8375,17 +8375,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -8624,17 +8624,17 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -8877,17 +8877,17 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -9130,17 +9130,17 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -9383,17 +9383,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -9632,17 +9632,17 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -9885,17 +9885,17 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -10138,17 +10138,17 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -10391,17 +10391,17 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -10644,17 +10644,17 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -10897,17 +10897,17 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -11150,17 +11150,17 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -11403,17 +11403,17 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -11656,17 +11656,17 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -11909,17 +11909,17 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -12162,17 +12162,17 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -12415,17 +12415,17 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -12668,17 +12668,17 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -12921,17 +12921,17 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -13174,17 +13174,17 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -13427,17 +13427,17 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -13680,17 +13680,17 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>TRATADO</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>111001098817</t>
+          <t>111001046931</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO NUEVA ROMA (IED)</t>
+          <t>COLEGIO ATABANZHA (IED)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">

</xml_diff>